<commit_message>
research and consultancy completed data update
</commit_message>
<xml_diff>
--- a/excels/Consultancy.xlsx
+++ b/excels/Consultancy.xlsx
@@ -29,9 +29,6 @@
     <t xml:space="preserve">S.No </t>
   </si>
   <si>
-    <t>Project Title -Broad Area</t>
-  </si>
-  <si>
     <t>Sponsored By</t>
   </si>
   <si>
@@ -92,9 +89,6 @@
     <t>Traffic Evaluation Demand Studies</t>
   </si>
   <si>
-    <t>Hyderabad Evaluation Studies Vijayawada</t>
-  </si>
-  <si>
     <t>Development of Expressway</t>
   </si>
   <si>
@@ -294,6 +288,12 @@
   </si>
   <si>
     <t>R&amp;B Department, Telangana</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Project Title-Broad Area</t>
   </si>
 </sst>
 </file>
@@ -632,10 +632,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -643,10 +643,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -654,10 +654,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -665,10 +665,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -676,10 +676,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -687,10 +687,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -698,10 +698,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -709,10 +709,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -720,10 +720,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -731,10 +731,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -742,10 +742,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -753,10 +753,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -764,10 +764,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -775,10 +775,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -786,10 +786,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -797,10 +797,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -808,10 +808,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="C17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -819,10 +819,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -830,10 +830,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C19" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -841,10 +841,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -852,10 +852,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -863,10 +863,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -874,10 +874,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -885,10 +885,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -896,10 +896,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -907,10 +907,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C26" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -918,10 +918,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C27" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -929,10 +929,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C28" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -940,10 +940,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C29" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -951,10 +951,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C30" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -962,10 +962,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C31" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -973,10 +973,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C32" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -984,10 +984,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -995,10 +995,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1006,10 +1006,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C35" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1017,10 +1017,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1028,10 +1028,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C37" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1039,10 +1039,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C38" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1050,10 +1050,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C39" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1061,10 +1061,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C40" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1072,10 +1072,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C41" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1083,10 +1083,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C42" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1094,10 +1094,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C43" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1105,10 +1105,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C44" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1116,10 +1116,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C45" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1127,10 +1127,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C46" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1138,10 +1138,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C47" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1149,10 +1149,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C48" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1160,10 +1160,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C49" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1171,10 +1171,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C50" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1182,10 +1182,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C51" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1193,10 +1193,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C52" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1204,10 +1204,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C53" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -1215,10 +1215,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C54" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
research and consultancy onging tab update
</commit_message>
<xml_diff>
--- a/excels/Consultancy.xlsx
+++ b/excels/Consultancy.xlsx
@@ -1,18 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\fmain\NITW-Transportation-Division-main\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A9A296-322A-47C0-8D83-B247B14D9F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="12150"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name=" Completed Consultancy" sheetId="1" r:id="rId1"/>
+    <sheet name="Ongoing Consultancy" sheetId="2" r:id="rId1"/>
+    <sheet name="Completed Consultancy" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="133">
   <si>
     <t xml:space="preserve">S.No </t>
   </si>
@@ -294,12 +296,141 @@
   </si>
   <si>
     <t>Project Title-Broad Area</t>
+  </si>
+  <si>
+    <t>Project_Title</t>
+  </si>
+  <si>
+    <t>Research_Domain</t>
+  </si>
+  <si>
+    <t>Technology_Used</t>
+  </si>
+  <si>
+    <t>Start_Date</t>
+  </si>
+  <si>
+    <t>Current_Status</t>
+  </si>
+  <si>
+    <t>Completion_Percentage</t>
+  </si>
+  <si>
+    <t>Team_Size</t>
+  </si>
+  <si>
+    <t>Funding_Amount_USD</t>
+  </si>
+  <si>
+    <t>ERP Implementation for Manufacturing Client</t>
+  </si>
+  <si>
+    <t>Enterprise Solutions</t>
+  </si>
+  <si>
+    <t>SAP S/4HANA, Fiori</t>
+  </si>
+  <si>
+    <t>Development</t>
+  </si>
+  <si>
+    <t>Cloud Migration Consultancy</t>
+  </si>
+  <si>
+    <t>Cloud Computing</t>
+  </si>
+  <si>
+    <t>AWS, Docker, Kubernetes</t>
+  </si>
+  <si>
+    <t>Deployment</t>
+  </si>
+  <si>
+    <t>Healthcare Data Analytics Consulting</t>
+  </si>
+  <si>
+    <t>Data Analytics</t>
+  </si>
+  <si>
+    <t>Power BI, Python, SQL</t>
+  </si>
+  <si>
+    <t>CRM Optimization Project</t>
+  </si>
+  <si>
+    <t>Business Intelligence</t>
+  </si>
+  <si>
+    <t>Salesforce, Apex</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>AI Customer Support Automation</t>
+  </si>
+  <si>
+    <t>Artificial Intelligence</t>
+  </si>
+  <si>
+    <t>OpenAI API, Python, NLP</t>
+  </si>
+  <si>
+    <t>Cybersecurity Risk Assessment</t>
+  </si>
+  <si>
+    <t>Cyber Security</t>
+  </si>
+  <si>
+    <t>SIEM, Wireshark, Kali Linux</t>
+  </si>
+  <si>
+    <t>Ongoing</t>
+  </si>
+  <si>
+    <t>Smart Inventory Management System</t>
+  </si>
+  <si>
+    <t>IoT &amp; Automation</t>
+  </si>
+  <si>
+    <t>RFID, NodeMCU, Firebase</t>
+  </si>
+  <si>
+    <t>Financial Forecasting Consultancy</t>
+  </si>
+  <si>
+    <t>FinTech</t>
+  </si>
+  <si>
+    <t>Tableau, Machine Learning</t>
+  </si>
+  <si>
+    <t>E-Learning Platform Enhancement</t>
+  </si>
+  <si>
+    <t>EdTech</t>
+  </si>
+  <si>
+    <t>React, Django, PostgreSQL</t>
+  </si>
+  <si>
+    <t>Planning</t>
+  </si>
+  <si>
+    <t>Digital Marketing Analytics Dashboard</t>
+  </si>
+  <si>
+    <t>Marketing Analytics</t>
+  </si>
+  <si>
+    <t>Google Analytics, Power BI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -337,9 +468,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -619,7 +759,311 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84D092AF-E5FD-451B-98A2-C562E36FCE67}">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D2" s="4">
+        <v>45672</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F2" s="3">
+        <v>68</v>
+      </c>
+      <c r="G2" s="3">
+        <v>8</v>
+      </c>
+      <c r="H2" s="3">
+        <v>52000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" s="4">
+        <v>45726</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" s="3">
+        <v>81</v>
+      </c>
+      <c r="G3" s="3">
+        <v>6</v>
+      </c>
+      <c r="H3" s="3">
+        <v>74500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D4" s="4">
+        <v>45693</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F4" s="3">
+        <v>59</v>
+      </c>
+      <c r="G4" s="3">
+        <v>5</v>
+      </c>
+      <c r="H4" s="3">
+        <v>38400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" s="4">
+        <v>45759</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="F5" s="3">
+        <v>72</v>
+      </c>
+      <c r="G5" s="3">
+        <v>4</v>
+      </c>
+      <c r="H5" s="3">
+        <v>26750</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6" s="4">
+        <v>45797</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F6" s="3">
+        <v>88</v>
+      </c>
+      <c r="G6" s="3">
+        <v>7</v>
+      </c>
+      <c r="H6" s="3">
+        <v>69300</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="4">
+        <v>45816</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="F7" s="3">
+        <v>43</v>
+      </c>
+      <c r="G7" s="3">
+        <v>5</v>
+      </c>
+      <c r="H7" s="3">
+        <v>31800</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" s="4">
+        <v>45839</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F8" s="3">
+        <v>54</v>
+      </c>
+      <c r="G8" s="3">
+        <v>6</v>
+      </c>
+      <c r="H8" s="3">
+        <v>41200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D9" s="4">
+        <v>45744</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F9" s="3">
+        <v>91</v>
+      </c>
+      <c r="G9" s="3">
+        <v>3</v>
+      </c>
+      <c r="H9" s="3">
+        <v>28600</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D10" s="4">
+        <v>45883</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="F10" s="3">
+        <v>27</v>
+      </c>
+      <c r="G10" s="3">
+        <v>5</v>
+      </c>
+      <c r="H10" s="3">
+        <v>35600</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D11" s="4">
+        <v>45905</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="F11" s="3">
+        <v>49</v>
+      </c>
+      <c r="G11" s="3">
+        <v>4</v>
+      </c>
+      <c r="H11" s="3">
+        <v>22150</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
fixed onging consultancy error
</commit_message>
<xml_diff>
--- a/excels/Consultancy.xlsx
+++ b/excels/Consultancy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A9A296-322A-47C0-8D83-B247B14D9F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6AD227C-57B6-4507-AA93-BF2F7536D6AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ongoing Consultancy" sheetId="2" r:id="rId1"/>
@@ -764,7 +764,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
completed consultancy data and contact us email update
</commit_message>
<xml_diff>
--- a/excels/Consultancy.xlsx
+++ b/excels/Consultancy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6AD227C-57B6-4507-AA93-BF2F7536D6AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCB3D21-E8F0-4261-81F0-CC6EF6397E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ongoing Consultancy" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="134">
   <si>
     <t xml:space="preserve">S.No </t>
   </si>
@@ -425,6 +425,9 @@
   </si>
   <si>
     <t>Google Analytics, Power BI</t>
+  </si>
+  <si>
+    <t>Year</t>
   </si>
 </sst>
 </file>
@@ -797,7 +800,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>98</v>
       </c>
@@ -927,7 +930,7 @@
         <v>69300</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>116</v>
       </c>
@@ -953,7 +956,7 @@
         <v>31800</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>120</v>
       </c>
@@ -979,7 +982,7 @@
         <v>41200</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>123</v>
       </c>
@@ -1064,14 +1067,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="70.140625" customWidth="1"/>
     <col min="3" max="3" width="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1081,8 +1084,11 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1093,7 +1099,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1104,7 +1110,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1115,7 +1121,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1126,7 +1132,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1137,7 +1143,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1148,7 +1154,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1159,7 +1165,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1170,7 +1176,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1181,7 +1187,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1192,7 +1198,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1203,7 +1209,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1214,7 +1220,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1225,7 +1231,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1236,7 +1242,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1667,5 +1673,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated collaboration data, outreach activity read more new page, research and consultancy data
</commit_message>
<xml_diff>
--- a/excels/Consultancy.xlsx
+++ b/excels/Consultancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCB3D21-E8F0-4261-81F0-CC6EF6397E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A3D629-6435-48C1-9754-D23071C97667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ongoing Consultancy" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="109">
   <si>
     <t xml:space="preserve">S.No </t>
   </si>
@@ -301,140 +301,65 @@
     <t>Project_Title</t>
   </si>
   <si>
-    <t>Research_Domain</t>
-  </si>
-  <si>
-    <t>Technology_Used</t>
-  </si>
-  <si>
     <t>Start_Date</t>
   </si>
   <si>
-    <t>Current_Status</t>
-  </si>
-  <si>
-    <t>Completion_Percentage</t>
-  </si>
-  <si>
-    <t>Team_Size</t>
-  </si>
-  <si>
-    <t>Funding_Amount_USD</t>
-  </si>
-  <si>
-    <t>ERP Implementation for Manufacturing Client</t>
-  </si>
-  <si>
-    <t>Enterprise Solutions</t>
-  </si>
-  <si>
-    <t>SAP S/4HANA, Fiori</t>
-  </si>
-  <si>
-    <t>Development</t>
-  </si>
-  <si>
-    <t>Cloud Migration Consultancy</t>
-  </si>
-  <si>
-    <t>Cloud Computing</t>
-  </si>
-  <si>
-    <t>AWS, Docker, Kubernetes</t>
-  </si>
-  <si>
-    <t>Deployment</t>
-  </si>
-  <si>
-    <t>Healthcare Data Analytics Consulting</t>
-  </si>
-  <si>
-    <t>Data Analytics</t>
-  </si>
-  <si>
-    <t>Power BI, Python, SQL</t>
-  </si>
-  <si>
-    <t>CRM Optimization Project</t>
-  </si>
-  <si>
-    <t>Business Intelligence</t>
-  </si>
-  <si>
-    <t>Salesforce, Apex</t>
-  </si>
-  <si>
-    <t>Testing</t>
-  </si>
-  <si>
-    <t>AI Customer Support Automation</t>
-  </si>
-  <si>
-    <t>Artificial Intelligence</t>
-  </si>
-  <si>
-    <t>OpenAI API, Python, NLP</t>
-  </si>
-  <si>
-    <t>Cybersecurity Risk Assessment</t>
-  </si>
-  <si>
-    <t>Cyber Security</t>
-  </si>
-  <si>
-    <t>SIEM, Wireshark, Kali Linux</t>
-  </si>
-  <si>
-    <t>Ongoing</t>
-  </si>
-  <si>
-    <t>Smart Inventory Management System</t>
-  </si>
-  <si>
-    <t>IoT &amp; Automation</t>
-  </si>
-  <si>
-    <t>RFID, NodeMCU, Firebase</t>
-  </si>
-  <si>
-    <t>Financial Forecasting Consultancy</t>
-  </si>
-  <si>
-    <t>FinTech</t>
-  </si>
-  <si>
-    <t>Tableau, Machine Learning</t>
-  </si>
-  <si>
-    <t>E-Learning Platform Enhancement</t>
-  </si>
-  <si>
-    <t>EdTech</t>
-  </si>
-  <si>
-    <t>React, Django, PostgreSQL</t>
-  </si>
-  <si>
-    <t>Planning</t>
-  </si>
-  <si>
-    <t>Digital Marketing Analytics Dashboard</t>
-  </si>
-  <si>
-    <t>Marketing Analytics</t>
-  </si>
-  <si>
-    <t>Google Analytics, Power BI</t>
-  </si>
-  <si>
     <t>Year</t>
+  </si>
+  <si>
+    <t>Consultancy_ID</t>
+  </si>
+  <si>
+    <t>Client_Name</t>
+  </si>
+  <si>
+    <t>Consultancy_Area</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Consultant_Team_Size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construction of 4-Lane Access-Controlled Greenfield Highway Section of Nh-163g (Khammam – Vijayawada) from Remidicherla Village at Design Ch. 280+200 Km to Jakkampudi Village (on NH-16) at Design Ch. 309+909 Km (Total Length 29.709 Km) under Other Economic Corridor (NH (O)) Programme on Hybrid Annuity Mode in The States of Telangana and Andhra Pradesh (Package-II)-Vetting Of Pavement Design </t>
+  </si>
+  <si>
+    <t>Nov, 2026</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar, Dr. Venkaiah Chowdary and Dr. R. Vishnu</t>
+  </si>
+  <si>
+    <t>Accident Analysis at Dahegaon Village Bus Stop, Telangana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. S.Shankar Y. Sudheer Kumar and Dr. Vishnu </t>
+  </si>
+  <si>
+    <t>Consultancy Services for Conducting a Technical Audit on Existing 4 lane Hyderabad -Bangalore  Section of NH44 from km89.000+to 124.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. S. Shankar and Dr KVR Ravi Shankar </t>
+  </si>
+  <si>
+    <t>Mix Desing for GSB Grade1 and Grade VI</t>
+  </si>
+  <si>
+    <t>Dr S. Shankar, Dr. Venkaiah Chowdary and Dr. R. Vishnu</t>
+  </si>
+  <si>
+    <t>Providing Proof Checking/Vetting for NICZISCL Zaheerabad Node, Telangana</t>
+  </si>
+  <si>
+    <t>Project_Value</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -446,6 +371,24 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -471,17 +414,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="17" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -766,301 +721,184 @@
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="53.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>94</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="D2" s="4"/>
+      <c r="E2" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="F2" s="3"/>
+      <c r="G2" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="D2" s="4">
-        <v>45672</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="H2" s="8">
+        <v>140400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="F2" s="3">
-        <v>68</v>
-      </c>
-      <c r="G2" s="3">
-        <v>8</v>
-      </c>
-      <c r="H2" s="3">
-        <v>52000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="D3" s="4"/>
+      <c r="E3" s="6">
+        <v>45992</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H3" s="3">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="6">
+        <v>46054</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D3" s="4">
-        <v>45726</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="H4" s="8">
+        <v>997600</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F3" s="3">
-        <v>81</v>
-      </c>
-      <c r="G3" s="3">
-        <v>6</v>
-      </c>
-      <c r="H3" s="3">
-        <v>74500</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="D5" s="4"/>
+      <c r="E5" s="6">
+        <v>46082</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="H5" s="8">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="D4" s="4">
-        <v>45693</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="F4" s="3">
-        <v>59</v>
-      </c>
-      <c r="G4" s="3">
-        <v>5</v>
-      </c>
-      <c r="H4" s="3">
-        <v>38400</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="D5" s="4">
-        <v>45759</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="F5" s="3">
-        <v>72</v>
-      </c>
-      <c r="G5" s="3">
-        <v>4</v>
-      </c>
-      <c r="H5" s="3">
-        <v>26750</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D6" s="4">
-        <v>45797</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="F6" s="3">
-        <v>88</v>
-      </c>
-      <c r="G6" s="3">
-        <v>7</v>
-      </c>
-      <c r="H6" s="3">
-        <v>69300</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="D7" s="4">
-        <v>45816</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="F7" s="3">
-        <v>43</v>
-      </c>
-      <c r="G7" s="3">
-        <v>5</v>
-      </c>
-      <c r="H7" s="3">
-        <v>31800</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="D8" s="4">
-        <v>45839</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="F8" s="3">
-        <v>54</v>
-      </c>
-      <c r="G8" s="3">
-        <v>6</v>
-      </c>
-      <c r="H8" s="3">
-        <v>41200</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="D9" s="4">
-        <v>45744</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="F9" s="3">
-        <v>91</v>
-      </c>
-      <c r="G9" s="3">
-        <v>3</v>
-      </c>
-      <c r="H9" s="3">
-        <v>28600</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="D10" s="4">
-        <v>45883</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="F10" s="3">
-        <v>27</v>
-      </c>
-      <c r="G10" s="3">
-        <v>5</v>
-      </c>
-      <c r="H10" s="3">
-        <v>35600</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D11" s="4">
-        <v>45905</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="F11" s="3">
-        <v>49</v>
-      </c>
-      <c r="G11" s="3">
-        <v>4</v>
-      </c>
-      <c r="H11" s="3">
-        <v>22150</v>
-      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="6">
+        <v>46174</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="H6" s="8">
+        <v>4248000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1085,7 +923,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>133</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
consultancy data update and increased capacity building per page count
</commit_message>
<xml_diff>
--- a/excels/Consultancy.xlsx
+++ b/excels/Consultancy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A3D629-6435-48C1-9754-D23071C97667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B70ACDD6-7942-4635-9C27-667197808279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ongoing Consultancy" sheetId="2" r:id="rId1"/>
@@ -26,10 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="109">
-  <si>
-    <t xml:space="preserve">S.No </t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="178">
   <si>
     <t>Sponsored By</t>
   </si>
@@ -43,78 +40,15 @@
     <t>SUTP Toolkit on Urban Road Traffic System</t>
   </si>
   <si>
-    <t>CRRI–SIP 30 – Development of Road User Cost Models for High Speed Corridors</t>
-  </si>
-  <si>
-    <t>Road Diversion Scheme at Tirupathi</t>
-  </si>
-  <si>
     <t>Warangal Traffic Management</t>
   </si>
   <si>
-    <t>Bridge Load Feasibility Analysis</t>
-  </si>
-  <si>
-    <t>Design of Station at Chittoor</t>
-  </si>
-  <si>
-    <t>Costing of Grade Separation</t>
-  </si>
-  <si>
-    <t>Location of Road Project</t>
-  </si>
-  <si>
-    <t>Location of Truck Terminals, Hyderabad</t>
-  </si>
-  <si>
-    <t>Design of Inland Traffic Analysis</t>
-  </si>
-  <si>
-    <t>Design of Traffic Port, Hyderabad</t>
-  </si>
-  <si>
-    <t>Evaluation of Street Lighting in Hyderabad</t>
-  </si>
-  <si>
-    <t>Hyderabad of Pavement System</t>
-  </si>
-  <si>
-    <t>Rail Passenger Demand Estimation Study</t>
-  </si>
-  <si>
     <t>Economic Feasibility of Light Rail Transit</t>
   </si>
   <si>
-    <t>Pavement Estimation Studies</t>
-  </si>
-  <si>
-    <t>Traffic Evaluation Demand Studies</t>
-  </si>
-  <si>
-    <t>Development of Expressway</t>
-  </si>
-  <si>
-    <t>Traffic Studies of Diversion Curves</t>
-  </si>
-  <si>
-    <t>DB-HATS II</t>
-  </si>
-  <si>
-    <t>Suburbs II</t>
-  </si>
-  <si>
-    <t>Pavement Rail Patronage in Hyderabad</t>
-  </si>
-  <si>
     <t>Roughness and Axle Load Spectrum Studies</t>
   </si>
   <si>
-    <t>DPR for a Package of NH-7 &amp; NH-31 Road</t>
-  </si>
-  <si>
-    <t>Technical Feasibility of Raipur Bypass</t>
-  </si>
-  <si>
     <t>Evaluation of Failures in Pavements</t>
   </si>
   <si>
@@ -136,51 +70,21 @@
     <t>Pavement Design and Third Party QC</t>
   </si>
   <si>
-    <t>TTD, Tirupathi</t>
-  </si>
-  <si>
-    <t>RMC, Warangal</t>
-  </si>
-  <si>
     <t>R&amp;B Dept.</t>
   </si>
   <si>
-    <t>HUDA, Warangal</t>
-  </si>
-  <si>
     <t>HUDA, Hyderabad</t>
   </si>
   <si>
-    <t>Traffic Dept.</t>
-  </si>
-  <si>
     <t>WMC, Warangal</t>
   </si>
   <si>
-    <t>HUDA, Dept.</t>
-  </si>
-  <si>
-    <t>HUDA Dept.</t>
-  </si>
-  <si>
-    <t>RITS</t>
-  </si>
-  <si>
-    <t>IL&amp;FS, New Delhi</t>
-  </si>
-  <si>
-    <t>STUP, Mumbai</t>
-  </si>
-  <si>
     <t>STUP, New Delhi</t>
   </si>
   <si>
     <t>MMRDA, Mumbai</t>
   </si>
   <si>
-    <t>KMCIT/DCL, R&amp;B Dept.</t>
-  </si>
-  <si>
     <t>Sheladia–PBI, AARVEE</t>
   </si>
   <si>
@@ -292,74 +196,377 @@
     <t>R&amp;B Department, Telangana</t>
   </si>
   <si>
-    <t>S</t>
+    <t>Project_Title</t>
+  </si>
+  <si>
+    <t>Start_Date</t>
+  </si>
+  <si>
+    <t>Consultant_Team_Size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construction of 4-Lane Access-Controlled Greenfield Highway Section of Nh-163g (Khammam – Vijayawada) from Remidicherla Village at Design Ch. 280+200 Km to Jakkampudi Village (on NH-16) at Design Ch. 309+909 Km (Total Length 29.709 Km) under Other Economic Corridor (NH (O)) Programme on Hybrid Annuity Mode in The States of Telangana and Andhra Pradesh (Package-II)-Vetting Of Pavement Design </t>
+  </si>
+  <si>
+    <t>Nov, 2026</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar, Dr. Venkaiah Chowdary and Dr. R. Vishnu</t>
+  </si>
+  <si>
+    <t>Accident Analysis at Dahegaon Village Bus Stop, Telangana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. S.Shankar Y. Sudheer Kumar and Dr. Vishnu </t>
+  </si>
+  <si>
+    <t>Consultancy Services for Conducting a Technical Audit on Existing 4 lane Hyderabad -Bangalore  Section of NH44 from km89.000+to 124.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. S. Shankar and Dr KVR Ravi Shankar </t>
+  </si>
+  <si>
+    <t>Mix Desing for GSB Grade1 and Grade VI</t>
+  </si>
+  <si>
+    <t>Dr S. Shankar, Dr. Venkaiah Chowdary and Dr. R. Vishnu</t>
+  </si>
+  <si>
+    <t>Providing Proof Checking/Vetting for NICZISCL Zaheerabad Node, Telangana</t>
+  </si>
+  <si>
+    <t>Project_Value</t>
+  </si>
+  <si>
+    <t>Estimation of Traffic Growth Rates at NORR</t>
+  </si>
+  <si>
+    <t> Vigilance and Enforcement Department and HMDA</t>
+  </si>
+  <si>
+    <t>GHMC Benefit Monitoring Evaluation Study of Flyovers/ Grade separators, Link Roads, and CRMP</t>
+  </si>
+  <si>
+    <t>Greater Hyderabad Municipal Corporation, Hyderabad</t>
+  </si>
+  <si>
+    <t>iRAP Star Rating of PWD North and North East zone Roads in the State of Karnataka under KSHIP-3</t>
+  </si>
+  <si>
+    <t>GeoVista-Government of Karnataka</t>
+  </si>
+  <si>
+    <t>2022 -23</t>
+  </si>
+  <si>
+    <t>Mahabubabad Junction Upgradation/Re-designs</t>
+  </si>
+  <si>
+    <t>Mahabubabad Municipal Corporation</t>
+  </si>
+  <si>
+    <t>Proof checking of short slab concrete pavement design</t>
+  </si>
+  <si>
+    <t>M/s. KPC Projects Ltd., IIPE Premises, Anakapalli, A.P.</t>
+  </si>
+  <si>
+    <t>Proof Checking / Vetting of Designs</t>
+  </si>
+  <si>
+    <t>May, 2026</t>
+  </si>
+  <si>
+    <t>Dr. S. Shankar</t>
+  </si>
+  <si>
+    <t>Forensic Investigtion of Flexible Pavement Construted with Terrazyme</t>
+  </si>
+  <si>
+    <t>Panchayt Raj Department, Government of Telanagna</t>
+  </si>
+  <si>
+    <t>Proof Checking of Pavement Design and Geometrics</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> GVPR/SRR JV-Telangana Industrial Infrastructure Corporation</t>
+  </si>
+  <si>
+    <t>Telangana power generation corporation limited BTPS (4 x 270 mw)- supply of permanent way material, PSC sleepers, ballast and linking of track for construction of railway siding and marshalling yard for BTPS, Manuguru, Bhadradri Kothagudem Dist-testing of ballast for finding out physical properties</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Private Agency</t>
+  </si>
+  <si>
+    <t>Construction of 6-lane Underpasses (4 No's) and allied works on existing 4 lane Hyderabad-Bangalore section of NH-44 from Km 89+000 to Km 124+000 in the State of Telangana on EPC mode, as part of Long-Term rectification of MoRTH identified Blackspots (TG-02-75, TG-02-97, TG-02-174 &amp; TG-02-59) - Providing Consultancy Services for conducting Technical Audit</t>
+  </si>
+  <si>
+    <t>National Highway Authority of India</t>
+  </si>
+  <si>
+    <t>Testing of dense bituminous macadam and bituminous concrete samples for resilient modulus, KMV Projects Ltd., Ameerpet, Hyderabad, Telangana</t>
+  </si>
+  <si>
+    <t>KMV Projects Ltd., Ameerpet, Hyderabad, Telangana</t>
+  </si>
+  <si>
+    <t>Full-depth reclamation Mix Design, samples supplied by Shri. Kale Narendra RamRao, Engineers and Contractors, Veejan Square, First Floor, Virat Hanuman Nagar, Rajiv Gandhi Chowk, Ausa Road, Latur-413512, Maharashtra</t>
+  </si>
+  <si>
+    <t>Road Agency , Maharashtra</t>
+  </si>
+  <si>
+    <t>Performance evaluation of roads constructed using waste plastic and conventional materials at reliance industries, Nagothane, Maharashtra</t>
+  </si>
+  <si>
+    <t>Reliance Industries, Mumbai through M/S Coact Solutions Hyd</t>
+  </si>
+  <si>
+    <t>Output and Performance based Road Contract for the Maintenance Roads under Package - 01 in Ernakulam, Kottayam, Alappuzha &amp; Pathanamthitta Districts of Kerala- material Testing</t>
+  </si>
+  <si>
+    <t>Private Agency ,Kerala</t>
+  </si>
+  <si>
+    <t>Widening and improvement of the existing carriageway to 2 lanes with paved shoulders from km86/160 to 121/730 of the jangaon- duddeda section of nh-365b in the state of telangana on an epc basis</t>
+  </si>
+  <si>
+    <t>NHAI</t>
+  </si>
+  <si>
+    <t>Providing Cement Concrete Roads at Food Storage Depot of Mancherial, Telangana</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Food Corporation of India (FCI), Mancherial, Mancherial Dist</t>
+  </si>
+  <si>
+    <t>Improvement of Runway by Resurfacing of Flexible Pavement and Allied Works at Air Force Station Bidar</t>
+  </si>
+  <si>
+    <t>Air Force Station, Bidar, Karnataka</t>
+  </si>
+  <si>
+    <t>Performance Evaluation of Four Roads Constructed using TerraZyme one each in the Chennur Block (AP04131405) and Pendlimarri Block (AP04131406) of YSR Kadapa District and Chillakur Block (AP141402) and Doravarisatram Block (AP141403) of Nellore District</t>
+  </si>
+  <si>
+    <t>Avijeet Agencies, Chennai, TamilNadu</t>
+  </si>
+  <si>
+    <t>2018-19</t>
+  </si>
+  <si>
+    <t>Traffic simulation study on Rajiv Gandhi International Airport roundabouts, Shamshabad</t>
+  </si>
+  <si>
+    <t>Sheladia Associates, Hyderabad</t>
+  </si>
+  <si>
+    <t>Extension and Resurfacing of Parade Ground and Associated Work Services</t>
+  </si>
+  <si>
+    <t>Air Force Academy, Dundigal, Hyderabad</t>
+  </si>
+  <si>
+    <t>Grading of Bitumen for Samples Collected from Four Hot Mix Plants during Quality Control Inspection</t>
+  </si>
+  <si>
+    <t>Roads and Buildings Department, Warangal</t>
+  </si>
+  <si>
+    <t>Third party quality checks for diversion road work and cross drainage works at RKOCP</t>
+  </si>
+  <si>
+    <t>Singareni Collieries Company Limited, Mandamarri, Adilabad</t>
+  </si>
+  <si>
+    <t>2015-16</t>
+  </si>
+  <si>
+    <t>Construction and Resurfacing of Various Roads</t>
+  </si>
+  <si>
+    <t>Singareni Collieries Company Limited, Bhupalpalli, Warangal</t>
+  </si>
+  <si>
+    <t>Renovation and Recarpeting of Internal Roads (Phase-I) for NIT at Warangal</t>
+  </si>
+  <si>
+    <t>Provision of Levelling and Resurfacing of Road</t>
+  </si>
+  <si>
+    <t>Central Public Works Department, Warangal, A.P.</t>
+  </si>
+  <si>
+    <t>2013-14</t>
+  </si>
+  <si>
+    <t>Road Safety Analysis of Accident at Meedikonda X Roads on NH 163</t>
+  </si>
+  <si>
+    <t>Telangana State Road Transport Corporation</t>
+  </si>
+  <si>
+    <t>Comprehensive Traffic Study for Karimnagar City</t>
+  </si>
+  <si>
+    <t>Municipal Corporation of Karimnagar, Telangana State</t>
+  </si>
+  <si>
+    <t>2017-19</t>
+  </si>
+  <si>
+    <t>Design of Traffic Junctions in Tirupati</t>
+  </si>
+  <si>
+    <t>Tirumala Tirupati Devasthanam (TTD), Andhra Pradesh</t>
+  </si>
+  <si>
+    <t>2017-18</t>
+  </si>
+  <si>
+    <t>DESIGN OF DENSE GRADED BITUMINOUS MIX INCORPORATING RECYCLED ASPHALT PAVEMENT (RAP) MATERIAL FOR THE STRENGTHENING AND WIDENING PROJECT BETWEEN BAMNI TO MH/TG BORDER (Ch 19+000 TO 51+985) OF NH-930D, MAHARASHTRA</t>
+  </si>
+  <si>
+    <t>G R infra Projects Ltd</t>
+  </si>
+  <si>
+    <t>REPAIR AND REHABILITATION STRATEGY OF NH163 (CHAINAGE 54+000 TO 153+103, BETWEEN YADAGIRI TO WARANGAL) IN TELANGANA STATE</t>
+  </si>
+  <si>
+    <t>FORENSIC INVESTIGATION OF SLIPPAGE FAILURE OF BITUMINOUS CONCRETE IN SH 148 BETWEEN CHAINAGE 26+400 TO 54+400 (SAMARLAKOTA TO RAJANAGARAM), ANDHRA PRADESH</t>
+  </si>
+  <si>
+    <t>Performance evaluation of low volume roads constructed with Terrazyme technology in Tamil Nadu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> M/S BSR BSCPL (JV)</t>
+  </si>
+  <si>
+    <t>Avajeet Agencies Pvt Ltd</t>
+  </si>
+  <si>
+    <t>Road Diversion Scheme at Tirupati</t>
+  </si>
+  <si>
+    <t>TTD, Tirupati</t>
+  </si>
+  <si>
+    <t>Bridge Location at Chittakodur</t>
+  </si>
+  <si>
+    <t>Design of Grade Separation Complex</t>
+  </si>
+  <si>
+    <t>Coastal Road Project–Feasibility Analysis</t>
+  </si>
+  <si>
+    <t>Location of Truck Terminals</t>
+  </si>
+  <si>
+    <t>KUDA, Warangal</t>
+  </si>
+  <si>
+    <t>Location of Inland Port, Hyderabad</t>
+  </si>
+  <si>
+    <t>Design of Traffic Signals in Hyderabad</t>
+  </si>
+  <si>
+    <t>Traffic Police, Hyderabad</t>
+  </si>
+  <si>
+    <t>Design of Street Lighting System</t>
+  </si>
+  <si>
+    <t>Evaluation of the Pavement Failures</t>
+  </si>
+  <si>
+    <t>Hyderabad Area Transportation Study</t>
+  </si>
+  <si>
+    <t>HUDA</t>
+  </si>
+  <si>
+    <t>Rail Passenger Demand Estimation</t>
+  </si>
+  <si>
+    <t>RITES, New Delhi</t>
+  </si>
+  <si>
+    <t>IL&amp;FS, Mumbai</t>
+  </si>
+  <si>
+    <t>Pavement Evaluation for Vijayawada</t>
+  </si>
+  <si>
+    <t>Traffic Estimation for Vijayawada Hyderabad Expressway</t>
+  </si>
+  <si>
+    <t>Development of Diversion Curves</t>
+  </si>
+  <si>
+    <t>Traffic Studies for Tirupati</t>
+  </si>
+  <si>
+    <t>DB–HATS II</t>
+  </si>
+  <si>
+    <t>Suburban Rail Patronage in Hyderabad</t>
+  </si>
+  <si>
+    <t>KMC/TDCL, R&amp;B Dept.</t>
+  </si>
+  <si>
+    <t>DPR for a Package of NH-7 &amp; NH-31</t>
+  </si>
+  <si>
+    <t>Technical Feasibility of Raipur Bypass Road</t>
+  </si>
+  <si>
+    <t>APSRTC, Hyderabad</t>
+  </si>
+  <si>
+    <t>SCCL, Kothagudem</t>
+  </si>
+  <si>
+    <t>Pavement Evaluation and Road Safety Audit</t>
+  </si>
+  <si>
+    <t>Simplex Infrastructures Ltd, Hyderabad</t>
+  </si>
+  <si>
+    <t>Roads &amp; Buildings Dept., Hyderabad, AP</t>
+  </si>
+  <si>
+    <t>CRRI–SIP 30–Development of Road User Cost Models for High Speed Corridors</t>
+  </si>
+  <si>
+    <t>CSIR-CRRI, New Delhi</t>
+  </si>
+  <si>
+    <t>IUT, MoUD, New Delhi</t>
+  </si>
+  <si>
+    <t>GeoVista, Hyderabad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year </t>
+  </si>
+  <si>
+    <t>PRED, GoAP, Hyderabad</t>
   </si>
   <si>
     <t>Project Title-Broad Area</t>
   </si>
   <si>
-    <t>Project_Title</t>
-  </si>
-  <si>
-    <t>Start_Date</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Consultancy_ID</t>
-  </si>
-  <si>
-    <t>Client_Name</t>
-  </si>
-  <si>
-    <t>Consultancy_Area</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Consultant_Team_Size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Construction of 4-Lane Access-Controlled Greenfield Highway Section of Nh-163g (Khammam – Vijayawada) from Remidicherla Village at Design Ch. 280+200 Km to Jakkampudi Village (on NH-16) at Design Ch. 309+909 Km (Total Length 29.709 Km) under Other Economic Corridor (NH (O)) Programme on Hybrid Annuity Mode in The States of Telangana and Andhra Pradesh (Package-II)-Vetting Of Pavement Design </t>
-  </si>
-  <si>
-    <t>Nov, 2026</t>
-  </si>
-  <si>
-    <t>Dr. S. Shankar, Dr. Venkaiah Chowdary and Dr. R. Vishnu</t>
-  </si>
-  <si>
-    <t>Accident Analysis at Dahegaon Village Bus Stop, Telangana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dr. S.Shankar Y. Sudheer Kumar and Dr. Vishnu </t>
-  </si>
-  <si>
-    <t>Consultancy Services for Conducting a Technical Audit on Existing 4 lane Hyderabad -Bangalore  Section of NH44 from km89.000+to 124.000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dr. S. Shankar and Dr KVR Ravi Shankar </t>
-  </si>
-  <si>
-    <t>Mix Desing for GSB Grade1 and Grade VI</t>
-  </si>
-  <si>
-    <t>Dr S. Shankar, Dr. Venkaiah Chowdary and Dr. R. Vishnu</t>
-  </si>
-  <si>
-    <t>Providing Proof Checking/Vetting for NICZISCL Zaheerabad Node, Telangana</t>
-  </si>
-  <si>
-    <t>Project_Value</t>
+    <t>S.No</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -393,6 +600,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -414,7 +628,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -437,6 +651,18 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -717,185 +943,143 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84D092AF-E5FD-451B-98A2-C562E36FCE67}">
-  <dimension ref="A1:H11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="72.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="72.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.28515625" customWidth="1"/>
+    <col min="3" max="3" width="53.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>93</v>
+        <v>56</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>82</v>
+      </c>
       <c r="C2" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="H2" s="8">
+        <v>83</v>
+      </c>
+      <c r="D2" s="3">
+        <v>42.48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="8">
         <v>140400</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="6">
+    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="6">
         <v>45992</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="H3" s="3">
+      <c r="C4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="3">
         <v>35000</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="6">
+    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="6">
         <v>46054</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="H4" s="8">
+      <c r="C5" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" s="8">
         <v>997600</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="6">
+    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="6">
         <v>46082</v>
       </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="H5" s="8">
+      <c r="C6" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="8">
         <v>60000</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="6">
+    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="6">
         <v>46174</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="H6" s="8">
+      <c r="C7" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="8">
         <v>4248000</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="3"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
+    <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="5"/>
       <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C8" s="5"/>
+      <c r="D8" s="3"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D9" s="3"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="D11" s="3"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -904,26 +1088,27 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D54"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="70.140625" customWidth="1"/>
-    <col min="3" max="3" width="37" customWidth="1"/>
+    <col min="3" max="3" width="37" style="10" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>92</v>
+      <c r="D1" s="9" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -931,10 +1116,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>36</v>
+        <v>139</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -942,10 +1127,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>37</v>
+        <v>4</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -953,10 +1138,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>38</v>
+        <v>141</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -964,10 +1149,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>38</v>
+        <v>142</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -975,10 +1160,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>38</v>
+        <v>143</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -986,10 +1171,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s">
-        <v>39</v>
+        <v>144</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -997,10 +1182,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" t="s">
-        <v>40</v>
+        <v>146</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1008,10 +1193,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" t="s">
-        <v>41</v>
+        <v>147</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1019,10 +1204,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" t="s">
-        <v>42</v>
+        <v>149</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1030,10 +1215,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" t="s">
-        <v>43</v>
+        <v>150</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1041,10 +1226,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" t="s">
-        <v>44</v>
+        <v>151</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1052,10 +1237,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" t="s">
-        <v>40</v>
+        <v>153</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1063,10 +1248,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" t="s">
-        <v>45</v>
+        <v>5</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1074,10 +1259,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
-      </c>
-      <c r="C15" t="s">
-        <v>42</v>
+        <v>156</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1085,10 +1270,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" t="s">
-        <v>44</v>
+        <v>157</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1096,10 +1281,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>88</v>
-      </c>
-      <c r="C17" t="s">
-        <v>44</v>
+        <v>158</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1107,10 +1292,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" t="s">
-        <v>40</v>
+        <v>159</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -1118,10 +1303,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" t="s">
-        <v>45</v>
+        <v>160</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1129,10 +1314,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" t="s">
-        <v>42</v>
+        <v>161</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1140,10 +1325,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" t="s">
-        <v>44</v>
+        <v>41</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1151,10 +1336,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
-      </c>
-      <c r="C22" t="s">
-        <v>46</v>
+        <v>6</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1162,10 +1347,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
-      </c>
-      <c r="C23" t="s">
-        <v>47</v>
+        <v>163</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1173,10 +1358,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" t="s">
-        <v>48</v>
+        <v>164</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1184,10 +1369,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" t="s">
-        <v>49</v>
+        <v>7</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1195,10 +1380,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>29</v>
-      </c>
-      <c r="C26" t="s">
-        <v>36</v>
+        <v>8</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1206,10 +1391,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>30</v>
-      </c>
-      <c r="C27" t="s">
-        <v>40</v>
+        <v>9</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1217,10 +1402,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>31</v>
-      </c>
-      <c r="C28" t="s">
-        <v>50</v>
+        <v>10</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1228,10 +1413,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>32</v>
-      </c>
-      <c r="C29" t="s">
-        <v>51</v>
+        <v>11</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1239,10 +1424,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>33</v>
-      </c>
-      <c r="C30" t="s">
-        <v>52</v>
+        <v>12</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1250,10 +1435,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>34</v>
-      </c>
-      <c r="C31" t="s">
-        <v>53</v>
+        <v>13</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1261,10 +1446,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>35</v>
-      </c>
-      <c r="C32" t="s">
-        <v>54</v>
+        <v>167</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1272,10 +1457,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>5</v>
-      </c>
-      <c r="C33" t="s">
-        <v>48</v>
+        <v>35</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1283,10 +1468,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>4</v>
-      </c>
-      <c r="C34" t="s">
-        <v>55</v>
+        <v>170</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1296,8 +1481,8 @@
       <c r="B35" t="s">
         <v>3</v>
       </c>
-      <c r="C35" t="s">
-        <v>56</v>
+      <c r="C35" s="10" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1307,8 +1492,8 @@
       <c r="B36" t="s">
         <v>2</v>
       </c>
-      <c r="C36" t="s">
-        <v>57</v>
+      <c r="C36" s="10" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1316,10 +1501,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>67</v>
-      </c>
-      <c r="C37" t="s">
-        <v>57</v>
+        <v>1</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1327,10 +1512,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>58</v>
-      </c>
-      <c r="C38" t="s">
-        <v>76</v>
+        <v>26</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1338,10 +1523,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>59</v>
-      </c>
-      <c r="C39" t="s">
-        <v>77</v>
+        <v>27</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1349,10 +1534,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>60</v>
-      </c>
-      <c r="C40" t="s">
-        <v>40</v>
+        <v>28</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1360,10 +1545,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>61</v>
-      </c>
-      <c r="C41" t="s">
-        <v>78</v>
+        <v>29</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1371,10 +1556,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>62</v>
-      </c>
-      <c r="C42" t="s">
-        <v>77</v>
+        <v>30</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1382,10 +1567,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>63</v>
-      </c>
-      <c r="C43" t="s">
-        <v>79</v>
+        <v>31</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1393,10 +1578,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>64</v>
-      </c>
-      <c r="C44" t="s">
-        <v>80</v>
+        <v>32</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1404,10 +1589,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>65</v>
-      </c>
-      <c r="C45" t="s">
-        <v>77</v>
+        <v>33</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1415,10 +1600,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>66</v>
-      </c>
-      <c r="C46" t="s">
-        <v>81</v>
+        <v>34</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1426,10 +1611,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>68</v>
-      </c>
-      <c r="C47" t="s">
-        <v>82</v>
+        <v>36</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1437,76 +1622,510 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>69</v>
-      </c>
-      <c r="C48" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>70</v>
-      </c>
-      <c r="C49" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>71</v>
-      </c>
-      <c r="C50" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>72</v>
-      </c>
-      <c r="C51" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C51" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>73</v>
-      </c>
-      <c r="C52" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="C52" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>74</v>
-      </c>
-      <c r="C53" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D53" s="10">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54" t="s">
+        <v>43</v>
+      </c>
+      <c r="C54" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>120</v>
+      </c>
+      <c r="C55" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>121</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D56" s="10">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>118</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D57" s="10">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>115</v>
+      </c>
+      <c r="C58" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D58" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>111</v>
+      </c>
+      <c r="C59" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D59" s="10">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>113</v>
+      </c>
+      <c r="C60" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="D60" s="10">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>129</v>
+      </c>
+      <c r="C61" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>126</v>
+      </c>
+      <c r="C62" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>109</v>
+      </c>
+      <c r="C63" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D63" s="10">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>106</v>
+      </c>
+      <c r="C64" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>104</v>
+      </c>
+      <c r="C65" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="D65" s="10">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>72</v>
+      </c>
+      <c r="C66" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D66" s="10">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>74</v>
+      </c>
+      <c r="C67" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D67" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>77</v>
+      </c>
+      <c r="C68" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D68" s="10">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>100</v>
+      </c>
+      <c r="C69" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D69" s="10">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>102</v>
+      </c>
+      <c r="C70" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D70" s="10">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>96</v>
+      </c>
+      <c r="C71" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D71" s="10">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>124</v>
+      </c>
+      <c r="C72" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D72" s="10">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>98</v>
+      </c>
+      <c r="C73" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="D73" s="10">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>92</v>
+      </c>
+      <c r="C74" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="D74" s="10">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>94</v>
+      </c>
+      <c r="C75" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="D75" s="10">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>70</v>
+      </c>
+      <c r="C76" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D76" s="10">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>136</v>
+      </c>
+      <c r="C77" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D77" s="10">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>88</v>
+      </c>
+      <c r="C78" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="D78" s="10">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>90</v>
+      </c>
+      <c r="C79" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="D79" s="10">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>79</v>
+      </c>
+      <c r="C80" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D80" s="10">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>132</v>
+      </c>
+      <c r="C81" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D81" s="10">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>134</v>
+      </c>
+      <c r="D82" s="10">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>135</v>
+      </c>
+      <c r="C83" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D83" s="10">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>84</v>
+      </c>
+      <c r="C84" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="D84" s="10">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>86</v>
+      </c>
+      <c r="C85" s="10" t="s">
         <v>87</v>
+      </c>
+      <c r="D85" s="10">
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
consultancy data update heading error
</commit_message>
<xml_diff>
--- a/excels/Consultancy.xlsx
+++ b/excels/Consultancy.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Documents\PA_catts(A)\mainnn\NITW-Transportation-Division-main\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7EDCE3F-2D28-4E6A-96FE-5951B3FF7132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="8550" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ongoing Consultancy" sheetId="2" r:id="rId1"/>
@@ -444,9 +445,6 @@
     <t>Avajeet Agencies Pvt Ltd</t>
   </si>
   <si>
-    <t>S.No.</t>
-  </si>
-  <si>
     <t>Road Diversion Scheme at Tirupati</t>
   </si>
   <si>
@@ -562,12 +560,15 @@
   </si>
   <si>
     <t>NHAI PIU Warangal</t>
+  </si>
+  <si>
+    <t>S.No</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -630,7 +631,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -659,9 +660,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -945,7 +943,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -970,16 +968,16 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="3">
         <v>42.48</v>
       </c>
     </row>
@@ -1090,7 +1088,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1101,16 +1099,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>177</v>
+        <v>178</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>176</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1118,10 +1116,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>140</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1140,7 +1138,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>14</v>
@@ -1151,7 +1149,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>14</v>
@@ -1162,7 +1160,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>14</v>
@@ -1173,10 +1171,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>145</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1184,7 +1182,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>15</v>
@@ -1195,10 +1193,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>147</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>148</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1206,7 +1204,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>16</v>
@@ -1217,7 +1215,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>14</v>
@@ -1228,10 +1226,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>151</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>152</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1239,10 +1237,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>153</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>154</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1253,7 +1251,7 @@
         <v>5</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1261,7 +1259,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>17</v>
@@ -1272,7 +1270,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C16" s="10" t="s">
         <v>15</v>
@@ -1283,7 +1281,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C17" s="10" t="s">
         <v>18</v>
@@ -1294,10 +1292,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -1305,7 +1303,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>15</v>
@@ -1316,7 +1314,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>15</v>
@@ -1330,7 +1328,7 @@
         <v>41</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1349,7 +1347,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>20</v>
@@ -1360,7 +1358,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C24" s="10" t="s">
         <v>21</v>
@@ -1385,7 +1383,7 @@
         <v>8</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1440,7 +1438,7 @@
         <v>13</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1448,10 +1446,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
+        <v>167</v>
+      </c>
+      <c r="C32" s="10" t="s">
         <v>168</v>
-      </c>
-      <c r="C32" s="10" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1462,7 +1460,7 @@
         <v>35</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1470,10 +1468,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
+        <v>170</v>
+      </c>
+      <c r="C34" s="10" t="s">
         <v>171</v>
-      </c>
-      <c r="C34" s="10" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1484,7 +1482,7 @@
         <v>3</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1495,7 +1493,7 @@
         <v>2</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1506,7 +1504,7 @@
         <v>1</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -2085,7 +2083,7 @@
         <v>134</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D82" s="10">
         <v>2026</v>

</xml_diff>